<commit_message>
Restore Aleksander Amundsen 10 km result with pacer note
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -3828,7 +3828,7 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Ole Jonas Nybø</t>
+          <t>Aleksander Amundsen</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>M40-44</t>
+          <t>M24-34</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -86691,7 +86691,7 @@
         <v>134</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>

</xml_diff>